<commit_message>
persist filters with url
</commit_message>
<xml_diff>
--- a/prisma/universities/Chungnam National University/1. 2027 GKS-U Available Departments(Chungnam National Univ).xlsx
+++ b/prisma/universities/Chungnam National University/1. 2027 GKS-U Available Departments(Chungnam National Univ).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\AppData\Local\Temp\_AZTMP1_\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\max\Desktop\projects\gks-universities\prisma\universities\Chungnam National University\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67F353C5-7F39-4D9D-ABD3-392B9055CF2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C1BA850-935C-4848-816D-FA251345092D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1BBC1D3F-468C-4CE6-8DA4-CF488D4DC87D}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="21600" windowHeight="13749" xr2:uid="{1BBC1D3F-468C-4CE6-8DA4-CF488D4DC87D}"/>
   </bookViews>
   <sheets>
     <sheet name=" Chungnam National University" sheetId="1" r:id="rId1"/>
@@ -23,9 +23,6 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -884,7 +881,7 @@
       <rPr>
         <sz val="9"/>
         <color theme="1"/>
-        <rFont val="맑은 고딕"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <charset val="129"/>
         <scheme val="minor"/>
@@ -968,11 +965,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -981,7 +978,7 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -996,7 +993,7 @@
     </font>
     <font>
       <sz val="8"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -1026,7 +1023,7 @@
       <u/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -1047,7 +1044,7 @@
     <font>
       <u/>
       <sz val="11"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -1063,7 +1060,7 @@
     <font>
       <sz val="9"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -1182,7 +1179,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1246,9 +1243,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1261,7 +1255,7 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1293,8 +1287,8 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="표준" xfId="0" builtinId="0"/>
-    <cellStyle name="하이퍼링크" xfId="1" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1310,9 +1304,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1350,7 +1344,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1456,7 +1450,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1598,7 +1592,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1607,106 +1601,106 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2F66D34-86C1-4AE9-B251-494C440601E1}">
   <dimension ref="A1:R41"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.3"/>
   <cols>
-    <col min="1" max="1" width="6.125" style="16" customWidth="1"/>
-    <col min="2" max="2" width="11.25" style="16" customWidth="1"/>
-    <col min="3" max="3" width="17.75" style="16" customWidth="1"/>
-    <col min="4" max="4" width="15.375" style="16" customWidth="1"/>
-    <col min="5" max="6" width="11.5" style="16" customWidth="1"/>
-    <col min="7" max="7" width="15.125" style="16" customWidth="1"/>
-    <col min="8" max="8" width="23.25" style="16" customWidth="1"/>
-    <col min="9" max="9" width="9.625" style="16" customWidth="1"/>
-    <col min="10" max="10" width="15.875" style="16" customWidth="1"/>
-    <col min="11" max="12" width="10.5" style="16" customWidth="1"/>
-    <col min="13" max="13" width="14.25" style="16" customWidth="1"/>
-    <col min="14" max="14" width="15.25" style="16" customWidth="1"/>
-    <col min="15" max="15" width="10.5" style="16" customWidth="1"/>
+    <col min="1" max="1" width="6.15234375" style="16" customWidth="1"/>
+    <col min="2" max="2" width="11.23046875" style="16" customWidth="1"/>
+    <col min="3" max="3" width="17.765625" style="16" customWidth="1"/>
+    <col min="4" max="4" width="15.3828125" style="16" customWidth="1"/>
+    <col min="5" max="6" width="11.4609375" style="16" customWidth="1"/>
+    <col min="7" max="7" width="15.15234375" style="16" customWidth="1"/>
+    <col min="8" max="8" width="23.23046875" style="16" customWidth="1"/>
+    <col min="9" max="9" width="9.61328125" style="16" customWidth="1"/>
+    <col min="10" max="10" width="15.84375" style="16" customWidth="1"/>
+    <col min="11" max="12" width="10.4609375" style="16" customWidth="1"/>
+    <col min="13" max="13" width="14.23046875" style="16" customWidth="1"/>
+    <col min="14" max="14" width="15.23046875" style="16" customWidth="1"/>
+    <col min="15" max="15" width="10.4609375" style="16" customWidth="1"/>
     <col min="16" max="16" width="31" style="16" customWidth="1"/>
     <col min="17" max="17" width="16" style="16" customWidth="1"/>
-    <col min="18" max="18" width="58.75" style="16" customWidth="1"/>
+    <col min="18" max="18" width="58.765625" style="16" customWidth="1"/>
     <col min="19" max="16384" width="9" style="16"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="41.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="33" t="s">
+    <row r="1" spans="1:18" ht="41.25" customHeight="1" thickBot="1">
+      <c r="A1" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="34"/>
-      <c r="J1" s="34"/>
-      <c r="K1" s="34"/>
-      <c r="L1" s="34"/>
-      <c r="M1" s="34"/>
-      <c r="N1" s="34"/>
-      <c r="O1" s="34"/>
-      <c r="P1" s="34"/>
-      <c r="Q1" s="34"/>
-      <c r="R1" s="35"/>
-    </row>
-    <row r="2" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="22" t="s">
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
+      <c r="J1" s="33"/>
+      <c r="K1" s="33"/>
+      <c r="L1" s="33"/>
+      <c r="M1" s="33"/>
+      <c r="N1" s="33"/>
+      <c r="O1" s="33"/>
+      <c r="P1" s="33"/>
+      <c r="Q1" s="33"/>
+      <c r="R1" s="34"/>
+    </row>
+    <row r="2" spans="1:18" ht="60.75" customHeight="1">
+      <c r="A2" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="22" t="s">
+      <c r="C2" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="22" t="s">
+      <c r="D2" s="21" t="s">
         <v>219</v>
       </c>
-      <c r="E2" s="22" t="s">
-        <v>4</v>
-      </c>
-      <c r="F2" s="22" t="s">
+      <c r="E2" s="21" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="22" t="s">
+      <c r="G2" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="22" t="s">
+      <c r="H2" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="30" t="s">
+      <c r="I2" s="29" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="30" t="s">
+      <c r="J2" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="29" t="s">
+      <c r="K2" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="29" t="s">
+      <c r="L2" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="M2" s="29" t="s">
+      <c r="M2" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="N2" s="29" t="s">
+      <c r="N2" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="O2" s="29" t="s">
+      <c r="O2" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="P2" s="22" t="s">
+      <c r="P2" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="Q2" s="22" t="s">
+      <c r="Q2" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="R2" s="22" t="s">
+      <c r="R2" s="21" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" ht="35.15" customHeight="1">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -1716,10 +1710,10 @@
       <c r="C3" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="28" t="s">
+      <c r="D3" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E3" s="23" t="s">
+      <c r="E3" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F3" s="1" t="s">
@@ -1731,25 +1725,25 @@
       <c r="H3" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I3" s="31" t="s">
+      <c r="I3" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="J3" s="31" t="s">
+      <c r="J3" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="K3" s="23" t="s">
+      <c r="K3" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="L3" s="23">
-        <v>4</v>
-      </c>
-      <c r="M3" s="23" t="s">
+      <c r="L3" s="22">
+        <v>4</v>
+      </c>
+      <c r="M3" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="N3" s="23" t="s">
+      <c r="N3" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="O3" s="23" t="s">
+      <c r="O3" s="22" t="s">
         <v>29</v>
       </c>
       <c r="P3" s="4" t="s">
@@ -1760,7 +1754,7 @@
       </c>
       <c r="R3" s="1"/>
     </row>
-    <row r="4" spans="1:18" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" ht="35.15" customHeight="1">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -1770,10 +1764,10 @@
       <c r="C4" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="28" t="s">
+      <c r="D4" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E4" s="23" t="s">
+      <c r="E4" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F4" s="1" t="s">
@@ -1785,25 +1779,25 @@
       <c r="H4" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="I4" s="31" t="s">
+      <c r="I4" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="J4" s="31" t="s">
+      <c r="J4" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="K4" s="23" t="s">
+      <c r="K4" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="L4" s="23">
-        <v>4</v>
-      </c>
-      <c r="M4" s="23" t="s">
+      <c r="L4" s="22">
+        <v>4</v>
+      </c>
+      <c r="M4" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="N4" s="23" t="s">
+      <c r="N4" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="O4" s="23" t="s">
+      <c r="O4" s="22" t="s">
         <v>29</v>
       </c>
       <c r="P4" s="4" t="s">
@@ -1814,7 +1808,7 @@
       </c>
       <c r="R4" s="1"/>
     </row>
-    <row r="5" spans="1:18" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" ht="35.15" customHeight="1">
       <c r="A5" s="1">
         <v>3</v>
       </c>
@@ -1824,10 +1818,10 @@
       <c r="C5" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D5" s="28" t="s">
+      <c r="D5" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E5" s="23" t="s">
+      <c r="E5" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F5" s="1" t="s">
@@ -1839,25 +1833,25 @@
       <c r="H5" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="I5" s="31" t="s">
+      <c r="I5" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="J5" s="31" t="s">
+      <c r="J5" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="K5" s="23" t="s">
+      <c r="K5" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="L5" s="23">
-        <v>4</v>
-      </c>
-      <c r="M5" s="23" t="s">
+      <c r="L5" s="22">
+        <v>4</v>
+      </c>
+      <c r="M5" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="N5" s="23" t="s">
+      <c r="N5" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="O5" s="23" t="s">
+      <c r="O5" s="22" t="s">
         <v>29</v>
       </c>
       <c r="P5" s="5" t="s">
@@ -1868,7 +1862,7 @@
       </c>
       <c r="R5" s="1"/>
     </row>
-    <row r="6" spans="1:18" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" ht="35.15" customHeight="1">
       <c r="A6" s="1">
         <v>4</v>
       </c>
@@ -1878,10 +1872,10 @@
       <c r="C6" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="28" t="s">
+      <c r="D6" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E6" s="23" t="s">
+      <c r="E6" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F6" s="1" t="s">
@@ -1893,25 +1887,25 @@
       <c r="H6" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="I6" s="31" t="s">
+      <c r="I6" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="J6" s="31" t="s">
+      <c r="J6" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="K6" s="23" t="s">
+      <c r="K6" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="L6" s="23">
-        <v>4</v>
-      </c>
-      <c r="M6" s="23" t="s">
+      <c r="L6" s="22">
+        <v>4</v>
+      </c>
+      <c r="M6" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="N6" s="23" t="s">
+      <c r="N6" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="O6" s="23" t="s">
+      <c r="O6" s="22" t="s">
         <v>29</v>
       </c>
       <c r="P6" s="4" t="s">
@@ -1922,7 +1916,7 @@
       </c>
       <c r="R6" s="1"/>
     </row>
-    <row r="7" spans="1:18" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" ht="35.15" customHeight="1">
       <c r="A7" s="1">
         <v>5</v>
       </c>
@@ -1932,10 +1926,10 @@
       <c r="C7" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="28" t="s">
+      <c r="D7" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E7" s="23" t="s">
+      <c r="E7" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F7" s="1" t="s">
@@ -1947,25 +1941,25 @@
       <c r="H7" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="I7" s="31" t="s">
+      <c r="I7" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="J7" s="31" t="s">
+      <c r="J7" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="K7" s="23" t="s">
+      <c r="K7" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="L7" s="23">
-        <v>4</v>
-      </c>
-      <c r="M7" s="23" t="s">
+      <c r="L7" s="22">
+        <v>4</v>
+      </c>
+      <c r="M7" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="N7" s="23" t="s">
+      <c r="N7" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="O7" s="23" t="s">
+      <c r="O7" s="22" t="s">
         <v>29</v>
       </c>
       <c r="P7" s="1" t="s">
@@ -1976,7 +1970,7 @@
       </c>
       <c r="R7" s="1"/>
     </row>
-    <row r="8" spans="1:18" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" ht="35.15" customHeight="1">
       <c r="A8" s="1">
         <v>6</v>
       </c>
@@ -1986,10 +1980,10 @@
       <c r="C8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="28" t="s">
+      <c r="D8" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E8" s="23" t="s">
+      <c r="E8" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F8" s="1" t="s">
@@ -2001,25 +1995,25 @@
       <c r="H8" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="I8" s="31" t="s">
+      <c r="I8" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="J8" s="31" t="s">
+      <c r="J8" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="K8" s="23" t="s">
+      <c r="K8" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="L8" s="23">
-        <v>4</v>
-      </c>
-      <c r="M8" s="23" t="s">
+      <c r="L8" s="22">
+        <v>4</v>
+      </c>
+      <c r="M8" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="N8" s="23" t="s">
+      <c r="N8" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="O8" s="23" t="s">
+      <c r="O8" s="22" t="s">
         <v>29</v>
       </c>
       <c r="P8" s="4" t="s">
@@ -2030,7 +2024,7 @@
       </c>
       <c r="R8" s="1"/>
     </row>
-    <row r="9" spans="1:18" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" ht="35.15" customHeight="1">
       <c r="A9" s="1">
         <v>7</v>
       </c>
@@ -2040,10 +2034,10 @@
       <c r="C9" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="28" t="s">
+      <c r="D9" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E9" s="23" t="s">
+      <c r="E9" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F9" s="1" t="s">
@@ -2055,25 +2049,25 @@
       <c r="H9" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="I9" s="31" t="s">
+      <c r="I9" s="30" t="s">
         <v>56</v>
       </c>
-      <c r="J9" s="31" t="s">
+      <c r="J9" s="30" t="s">
         <v>57</v>
       </c>
-      <c r="K9" s="23" t="s">
+      <c r="K9" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="L9" s="23">
-        <v>4</v>
-      </c>
-      <c r="M9" s="23" t="s">
+      <c r="L9" s="22">
+        <v>4</v>
+      </c>
+      <c r="M9" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="N9" s="23" t="s">
+      <c r="N9" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="O9" s="23" t="s">
+      <c r="O9" s="22" t="s">
         <v>29</v>
       </c>
       <c r="P9" s="4" t="s">
@@ -2084,7 +2078,7 @@
       </c>
       <c r="R9" s="1"/>
     </row>
-    <row r="10" spans="1:18" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" ht="35.15" customHeight="1">
       <c r="A10" s="1">
         <v>8</v>
       </c>
@@ -2094,10 +2088,10 @@
       <c r="C10" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D10" s="28" t="s">
+      <c r="D10" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E10" s="23" t="s">
+      <c r="E10" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F10" s="1" t="s">
@@ -2109,25 +2103,25 @@
       <c r="H10" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="I10" s="31" t="s">
+      <c r="I10" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="J10" s="31" t="s">
+      <c r="J10" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="K10" s="23" t="s">
+      <c r="K10" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="L10" s="23">
-        <v>4</v>
-      </c>
-      <c r="M10" s="23" t="s">
+      <c r="L10" s="22">
+        <v>4</v>
+      </c>
+      <c r="M10" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="N10" s="23" t="s">
+      <c r="N10" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="O10" s="23" t="s">
+      <c r="O10" s="22" t="s">
         <v>29</v>
       </c>
       <c r="P10" s="9" t="s">
@@ -2138,7 +2132,7 @@
       </c>
       <c r="R10" s="1"/>
     </row>
-    <row r="11" spans="1:18" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" ht="35.15" customHeight="1">
       <c r="A11" s="1">
         <v>9</v>
       </c>
@@ -2148,10 +2142,10 @@
       <c r="C11" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="28" t="s">
+      <c r="D11" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E11" s="23" t="s">
+      <c r="E11" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F11" s="1" t="s">
@@ -2163,25 +2157,25 @@
       <c r="H11" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="I11" s="31" t="s">
+      <c r="I11" s="30" t="s">
         <v>79</v>
       </c>
-      <c r="J11" s="31" t="s">
+      <c r="J11" s="30" t="s">
         <v>221</v>
       </c>
-      <c r="K11" s="23" t="s">
+      <c r="K11" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="L11" s="23">
-        <v>4</v>
-      </c>
-      <c r="M11" s="23" t="s">
+      <c r="L11" s="22">
+        <v>4</v>
+      </c>
+      <c r="M11" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="N11" s="23" t="s">
+      <c r="N11" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="O11" s="23" t="s">
+      <c r="O11" s="22" t="s">
         <v>29</v>
       </c>
       <c r="P11" s="4" t="s">
@@ -2192,7 +2186,7 @@
       </c>
       <c r="R11" s="1"/>
     </row>
-    <row r="12" spans="1:18" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" ht="35.15" customHeight="1">
       <c r="A12" s="1">
         <v>10</v>
       </c>
@@ -2202,10 +2196,10 @@
       <c r="C12" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D12" s="28" t="s">
+      <c r="D12" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E12" s="23" t="s">
+      <c r="E12" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F12" s="1" t="s">
@@ -2217,25 +2211,25 @@
       <c r="H12" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="I12" s="31" t="s">
+      <c r="I12" s="30" t="s">
         <v>79</v>
       </c>
-      <c r="J12" s="31" t="s">
+      <c r="J12" s="30" t="s">
         <v>221</v>
       </c>
-      <c r="K12" s="23" t="s">
+      <c r="K12" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="L12" s="23">
-        <v>4</v>
-      </c>
-      <c r="M12" s="23" t="s">
+      <c r="L12" s="22">
+        <v>4</v>
+      </c>
+      <c r="M12" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="N12" s="23" t="s">
+      <c r="N12" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="O12" s="23" t="s">
+      <c r="O12" s="22" t="s">
         <v>29</v>
       </c>
       <c r="P12" s="1" t="s">
@@ -2246,7 +2240,7 @@
       </c>
       <c r="R12" s="1"/>
     </row>
-    <row r="13" spans="1:18" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" ht="35.15" customHeight="1">
       <c r="A13" s="1">
         <v>11</v>
       </c>
@@ -2256,10 +2250,10 @@
       <c r="C13" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D13" s="28" t="s">
+      <c r="D13" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E13" s="23" t="s">
+      <c r="E13" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F13" s="1" t="s">
@@ -2271,25 +2265,25 @@
       <c r="H13" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="I13" s="31" t="s">
+      <c r="I13" s="30" t="s">
         <v>69</v>
       </c>
-      <c r="J13" s="31" t="s">
+      <c r="J13" s="30" t="s">
         <v>221</v>
       </c>
-      <c r="K13" s="23" t="s">
+      <c r="K13" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="L13" s="23">
-        <v>4</v>
-      </c>
-      <c r="M13" s="23" t="s">
+      <c r="L13" s="22">
+        <v>4</v>
+      </c>
+      <c r="M13" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="N13" s="23" t="s">
+      <c r="N13" s="22" t="s">
         <v>71</v>
       </c>
-      <c r="O13" s="23" t="s">
+      <c r="O13" s="22" t="s">
         <v>72</v>
       </c>
       <c r="P13" s="4" t="s">
@@ -2302,7 +2296,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="14" spans="1:18" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:18" ht="35.15" customHeight="1">
       <c r="A14" s="1">
         <v>12</v>
       </c>
@@ -2312,10 +2306,10 @@
       <c r="C14" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D14" s="28" t="s">
+      <c r="D14" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E14" s="23" t="s">
+      <c r="E14" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F14" s="1" t="s">
@@ -2327,25 +2321,25 @@
       <c r="H14" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="I14" s="31" t="s">
+      <c r="I14" s="30" t="s">
         <v>79</v>
       </c>
-      <c r="J14" s="31" t="s">
+      <c r="J14" s="30" t="s">
         <v>221</v>
       </c>
-      <c r="K14" s="23" t="s">
+      <c r="K14" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="L14" s="23">
-        <v>4</v>
-      </c>
-      <c r="M14" s="23" t="s">
+      <c r="L14" s="22">
+        <v>4</v>
+      </c>
+      <c r="M14" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="N14" s="23" t="s">
+      <c r="N14" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="O14" s="23" t="s">
+      <c r="O14" s="22" t="s">
         <v>29</v>
       </c>
       <c r="P14" s="4" t="s">
@@ -2356,7 +2350,7 @@
       </c>
       <c r="R14" s="1"/>
     </row>
-    <row r="15" spans="1:18" ht="346.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" ht="346.5" customHeight="1">
       <c r="A15" s="1">
         <v>13</v>
       </c>
@@ -2366,10 +2360,10 @@
       <c r="C15" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D15" s="28" t="s">
+      <c r="D15" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E15" s="23" t="s">
+      <c r="E15" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F15" s="1" t="s">
@@ -2381,25 +2375,25 @@
       <c r="H15" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="I15" s="31" t="s">
+      <c r="I15" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="J15" s="31" t="s">
+      <c r="J15" s="30" t="s">
         <v>85</v>
       </c>
-      <c r="K15" s="23" t="s">
+      <c r="K15" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="L15" s="23">
-        <v>4</v>
-      </c>
-      <c r="M15" s="23" t="s">
+      <c r="L15" s="22">
+        <v>4</v>
+      </c>
+      <c r="M15" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="N15" s="24" t="s">
+      <c r="N15" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="O15" s="23" t="s">
+      <c r="O15" s="22" t="s">
         <v>29</v>
       </c>
       <c r="P15" s="1" t="s">
@@ -2408,11 +2402,11 @@
       <c r="Q15" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="R15" s="26" t="s">
+      <c r="R15" s="25" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="16" spans="1:18" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:18" ht="35.15" customHeight="1">
       <c r="A16" s="1">
         <v>14</v>
       </c>
@@ -2422,10 +2416,10 @@
       <c r="C16" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D16" s="28" t="s">
+      <c r="D16" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E16" s="23" t="s">
+      <c r="E16" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F16" s="1" t="s">
@@ -2437,25 +2431,25 @@
       <c r="H16" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="I16" s="31" t="s">
+      <c r="I16" s="30" t="s">
         <v>176</v>
       </c>
-      <c r="J16" s="31" t="s">
+      <c r="J16" s="30" t="s">
         <v>177</v>
       </c>
-      <c r="K16" s="23" t="s">
+      <c r="K16" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="L16" s="23">
-        <v>4</v>
-      </c>
-      <c r="M16" s="23" t="s">
+      <c r="L16" s="22">
+        <v>4</v>
+      </c>
+      <c r="M16" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="N16" s="23" t="s">
+      <c r="N16" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="O16" s="23" t="s">
+      <c r="O16" s="22" t="s">
         <v>178</v>
       </c>
       <c r="P16" s="17" t="s">
@@ -2466,7 +2460,7 @@
       </c>
       <c r="R16" s="1"/>
     </row>
-    <row r="17" spans="1:18" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:18" ht="35.15" customHeight="1">
       <c r="A17" s="1">
         <v>15</v>
       </c>
@@ -2476,10 +2470,10 @@
       <c r="C17" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D17" s="28" t="s">
+      <c r="D17" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E17" s="23" t="s">
+      <c r="E17" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F17" s="1" t="s">
@@ -2491,25 +2485,25 @@
       <c r="H17" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="I17" s="31" t="s">
+      <c r="I17" s="30" t="s">
         <v>176</v>
       </c>
-      <c r="J17" s="31" t="s">
+      <c r="J17" s="30" t="s">
         <v>177</v>
       </c>
-      <c r="K17" s="23" t="s">
+      <c r="K17" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="L17" s="23">
-        <v>4</v>
-      </c>
-      <c r="M17" s="23" t="s">
+      <c r="L17" s="22">
+        <v>4</v>
+      </c>
+      <c r="M17" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="N17" s="23" t="s">
+      <c r="N17" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="O17" s="23" t="s">
+      <c r="O17" s="22" t="s">
         <v>183</v>
       </c>
       <c r="P17" s="4" t="s">
@@ -2520,7 +2514,7 @@
       </c>
       <c r="R17" s="1"/>
     </row>
-    <row r="18" spans="1:18" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:18" ht="35.15" customHeight="1">
       <c r="A18" s="1">
         <v>16</v>
       </c>
@@ -2530,10 +2524,10 @@
       <c r="C18" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D18" s="28" t="s">
+      <c r="D18" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E18" s="23" t="s">
+      <c r="E18" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F18" s="1" t="s">
@@ -2545,25 +2539,25 @@
       <c r="H18" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="I18" s="31" t="s">
+      <c r="I18" s="30" t="s">
         <v>188</v>
       </c>
-      <c r="J18" s="31" t="s">
+      <c r="J18" s="30" t="s">
         <v>177</v>
       </c>
-      <c r="K18" s="23" t="s">
+      <c r="K18" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="L18" s="23">
-        <v>4</v>
-      </c>
-      <c r="M18" s="23" t="s">
+      <c r="L18" s="22">
+        <v>4</v>
+      </c>
+      <c r="M18" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="N18" s="23" t="s">
+      <c r="N18" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="O18" s="23" t="s">
+      <c r="O18" s="22" t="s">
         <v>178</v>
       </c>
       <c r="P18" s="19" t="s">
@@ -2574,7 +2568,7 @@
       </c>
       <c r="R18" s="1"/>
     </row>
-    <row r="19" spans="1:18" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:18" ht="35.15" customHeight="1">
       <c r="A19" s="1">
         <v>17</v>
       </c>
@@ -2584,10 +2578,10 @@
       <c r="C19" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D19" s="28" t="s">
+      <c r="D19" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E19" s="23" t="s">
+      <c r="E19" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F19" s="1" t="s">
@@ -2599,25 +2593,25 @@
       <c r="H19" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="I19" s="31" t="s">
+      <c r="I19" s="30" t="s">
         <v>188</v>
       </c>
-      <c r="J19" s="31" t="s">
+      <c r="J19" s="30" t="s">
         <v>177</v>
       </c>
-      <c r="K19" s="23" t="s">
+      <c r="K19" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="L19" s="23">
-        <v>4</v>
-      </c>
-      <c r="M19" s="23" t="s">
+      <c r="L19" s="22">
+        <v>4</v>
+      </c>
+      <c r="M19" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="N19" s="23" t="s">
+      <c r="N19" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="O19" s="23" t="s">
+      <c r="O19" s="22" t="s">
         <v>178</v>
       </c>
       <c r="P19" s="4" t="s">
@@ -2628,7 +2622,7 @@
       </c>
       <c r="R19" s="1"/>
     </row>
-    <row r="20" spans="1:18" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:18" ht="35.15" customHeight="1">
       <c r="A20" s="1">
         <v>18</v>
       </c>
@@ -2638,10 +2632,10 @@
       <c r="C20" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D20" s="28" t="s">
+      <c r="D20" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E20" s="23" t="s">
+      <c r="E20" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F20" s="1" t="s">
@@ -2653,25 +2647,25 @@
       <c r="H20" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="I20" s="31" t="s">
+      <c r="I20" s="30" t="s">
         <v>188</v>
       </c>
-      <c r="J20" s="31" t="s">
+      <c r="J20" s="30" t="s">
         <v>177</v>
       </c>
-      <c r="K20" s="23" t="s">
+      <c r="K20" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="L20" s="23">
-        <v>4</v>
-      </c>
-      <c r="M20" s="23" t="s">
+      <c r="L20" s="22">
+        <v>4</v>
+      </c>
+      <c r="M20" s="22" t="s">
         <v>226</v>
       </c>
-      <c r="N20" s="23" t="s">
+      <c r="N20" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="O20" s="23" t="s">
+      <c r="O20" s="22" t="s">
         <v>178</v>
       </c>
       <c r="P20" s="17" t="s">
@@ -2682,7 +2676,7 @@
       </c>
       <c r="R20" s="1"/>
     </row>
-    <row r="21" spans="1:18" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:18" ht="35.15" customHeight="1">
       <c r="A21" s="1">
         <v>19</v>
       </c>
@@ -2692,10 +2686,10 @@
       <c r="C21" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D21" s="28" t="s">
+      <c r="D21" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E21" s="23" t="s">
+      <c r="E21" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F21" s="1" t="s">
@@ -2707,25 +2701,25 @@
       <c r="H21" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="I21" s="31" t="s">
+      <c r="I21" s="30" t="s">
         <v>188</v>
       </c>
-      <c r="J21" s="31" t="s">
+      <c r="J21" s="30" t="s">
         <v>177</v>
       </c>
-      <c r="K21" s="23" t="s">
+      <c r="K21" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="L21" s="23">
-        <v>4</v>
-      </c>
-      <c r="M21" s="25" t="s">
+      <c r="L21" s="22">
+        <v>4</v>
+      </c>
+      <c r="M21" s="24" t="s">
         <v>227</v>
       </c>
-      <c r="N21" s="23" t="s">
+      <c r="N21" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="O21" s="23" t="s">
+      <c r="O21" s="22" t="s">
         <v>72</v>
       </c>
       <c r="P21" s="20" t="s">
@@ -2736,7 +2730,7 @@
       </c>
       <c r="R21" s="1"/>
     </row>
-    <row r="22" spans="1:18" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:18" ht="35.15" customHeight="1">
       <c r="A22" s="1">
         <v>20</v>
       </c>
@@ -2746,10 +2740,10 @@
       <c r="C22" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D22" s="28" t="s">
+      <c r="D22" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E22" s="23" t="s">
+      <c r="E22" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F22" s="1" t="s">
@@ -2761,25 +2755,25 @@
       <c r="H22" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="I22" s="31" t="s">
+      <c r="I22" s="30" t="s">
         <v>188</v>
       </c>
-      <c r="J22" s="31" t="s">
+      <c r="J22" s="30" t="s">
         <v>177</v>
       </c>
-      <c r="K22" s="23" t="s">
+      <c r="K22" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="L22" s="23">
-        <v>4</v>
-      </c>
-      <c r="M22" s="23" t="s">
+      <c r="L22" s="22">
+        <v>4</v>
+      </c>
+      <c r="M22" s="22" t="s">
         <v>205</v>
       </c>
-      <c r="N22" s="23" t="s">
+      <c r="N22" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="O22" s="23" t="s">
+      <c r="O22" s="22" t="s">
         <v>178</v>
       </c>
       <c r="P22" s="1" t="s">
@@ -2790,7 +2784,7 @@
       </c>
       <c r="R22" s="1"/>
     </row>
-    <row r="23" spans="1:18" ht="27" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:18" ht="39.9">
       <c r="A23" s="1">
         <v>21</v>
       </c>
@@ -2800,10 +2794,10 @@
       <c r="C23" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D23" s="28" t="s">
+      <c r="D23" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E23" s="23" t="s">
+      <c r="E23" s="22" t="s">
         <v>208</v>
       </c>
       <c r="F23" s="1" t="s">
@@ -2815,25 +2809,25 @@
       <c r="H23" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="I23" s="31" t="s">
+      <c r="I23" s="30" t="s">
         <v>188</v>
       </c>
-      <c r="J23" s="31" t="s">
+      <c r="J23" s="30" t="s">
         <v>177</v>
       </c>
-      <c r="K23" s="23" t="s">
+      <c r="K23" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="L23" s="23">
-        <v>4</v>
-      </c>
-      <c r="M23" s="23" t="s">
+      <c r="L23" s="22">
+        <v>4</v>
+      </c>
+      <c r="M23" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="N23" s="23" t="s">
+      <c r="N23" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="O23" s="23" t="s">
+      <c r="O23" s="22" t="s">
         <v>178</v>
       </c>
       <c r="P23" s="1" t="s">
@@ -2844,7 +2838,7 @@
       </c>
       <c r="R23" s="1"/>
     </row>
-    <row r="24" spans="1:18" ht="27" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:18" ht="39.9">
       <c r="A24" s="1">
         <v>22</v>
       </c>
@@ -2854,10 +2848,10 @@
       <c r="C24" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D24" s="28" t="s">
+      <c r="D24" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E24" s="23" t="s">
+      <c r="E24" s="22" t="s">
         <v>208</v>
       </c>
       <c r="F24" s="1" t="s">
@@ -2869,25 +2863,25 @@
       <c r="H24" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="I24" s="31" t="s">
+      <c r="I24" s="30" t="s">
         <v>188</v>
       </c>
-      <c r="J24" s="31" t="s">
+      <c r="J24" s="30" t="s">
         <v>177</v>
       </c>
-      <c r="K24" s="23" t="s">
+      <c r="K24" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="L24" s="23">
-        <v>4</v>
-      </c>
-      <c r="M24" s="23" t="s">
+      <c r="L24" s="22">
+        <v>4</v>
+      </c>
+      <c r="M24" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="N24" s="23" t="s">
+      <c r="N24" s="22" t="s">
         <v>167</v>
       </c>
-      <c r="O24" s="23" t="s">
+      <c r="O24" s="22" t="s">
         <v>178</v>
       </c>
       <c r="P24" s="1" t="s">
@@ -2898,7 +2892,7 @@
       </c>
       <c r="R24" s="1"/>
     </row>
-    <row r="25" spans="1:18" ht="27" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:18" ht="39.9">
       <c r="A25" s="1">
         <v>23</v>
       </c>
@@ -2908,10 +2902,10 @@
       <c r="C25" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D25" s="28" t="s">
+      <c r="D25" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E25" s="23" t="s">
+      <c r="E25" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F25" s="1" t="s">
@@ -2923,25 +2917,25 @@
       <c r="H25" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="I25" s="31" t="s">
+      <c r="I25" s="30" t="s">
         <v>116</v>
       </c>
-      <c r="J25" s="31" t="s">
+      <c r="J25" s="30" t="s">
         <v>223</v>
       </c>
-      <c r="K25" s="23" t="s">
+      <c r="K25" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="L25" s="23">
-        <v>4</v>
-      </c>
-      <c r="M25" s="23" t="s">
+      <c r="L25" s="22">
+        <v>4</v>
+      </c>
+      <c r="M25" s="22" t="s">
         <v>228</v>
       </c>
-      <c r="N25" s="23" t="s">
+      <c r="N25" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="O25" s="23" t="s">
+      <c r="O25" s="22" t="s">
         <v>93</v>
       </c>
       <c r="P25" s="13" t="s">
@@ -2952,7 +2946,7 @@
       </c>
       <c r="R25" s="1"/>
     </row>
-    <row r="26" spans="1:18" ht="27" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:18" ht="39.9">
       <c r="A26" s="1">
         <v>24</v>
       </c>
@@ -2962,10 +2956,10 @@
       <c r="C26" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D26" s="28" t="s">
+      <c r="D26" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E26" s="23" t="s">
+      <c r="E26" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F26" s="1" t="s">
@@ -2977,25 +2971,25 @@
       <c r="H26" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="I26" s="31" t="s">
+      <c r="I26" s="30" t="s">
         <v>92</v>
       </c>
-      <c r="J26" s="31" t="s">
+      <c r="J26" s="30" t="s">
         <v>222</v>
       </c>
-      <c r="K26" s="23" t="s">
+      <c r="K26" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="L26" s="23">
-        <v>4</v>
-      </c>
-      <c r="M26" s="23" t="s">
+      <c r="L26" s="22">
+        <v>4</v>
+      </c>
+      <c r="M26" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="N26" s="23" t="s">
+      <c r="N26" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="O26" s="23" t="s">
+      <c r="O26" s="22" t="s">
         <v>29</v>
       </c>
       <c r="P26" s="4" t="s">
@@ -3006,7 +3000,7 @@
       </c>
       <c r="R26" s="1"/>
     </row>
-    <row r="27" spans="1:18" ht="27" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:18" ht="39.9">
       <c r="A27" s="1">
         <v>25</v>
       </c>
@@ -3016,10 +3010,10 @@
       <c r="C27" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D27" s="28" t="s">
+      <c r="D27" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E27" s="23" t="s">
+      <c r="E27" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F27" s="1" t="s">
@@ -3031,25 +3025,25 @@
       <c r="H27" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="I27" s="31" t="s">
+      <c r="I27" s="30" t="s">
         <v>116</v>
       </c>
-      <c r="J27" s="31" t="s">
+      <c r="J27" s="30" t="s">
         <v>223</v>
       </c>
-      <c r="K27" s="23" t="s">
+      <c r="K27" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="L27" s="23">
-        <v>4</v>
-      </c>
-      <c r="M27" s="23" t="s">
+      <c r="L27" s="22">
+        <v>4</v>
+      </c>
+      <c r="M27" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="N27" s="23" t="s">
+      <c r="N27" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="O27" s="23" t="s">
+      <c r="O27" s="22" t="s">
         <v>29</v>
       </c>
       <c r="P27" s="1" t="s">
@@ -3060,7 +3054,7 @@
       </c>
       <c r="R27" s="1"/>
     </row>
-    <row r="28" spans="1:18" ht="27" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:18" ht="39.9">
       <c r="A28" s="1">
         <v>26</v>
       </c>
@@ -3070,10 +3064,10 @@
       <c r="C28" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D28" s="28" t="s">
+      <c r="D28" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E28" s="23" t="s">
+      <c r="E28" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F28" s="1" t="s">
@@ -3085,25 +3079,25 @@
       <c r="H28" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="I28" s="31" t="s">
+      <c r="I28" s="30" t="s">
         <v>129</v>
       </c>
-      <c r="J28" s="31" t="s">
+      <c r="J28" s="30" t="s">
         <v>223</v>
       </c>
-      <c r="K28" s="23" t="s">
+      <c r="K28" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="L28" s="23">
-        <v>4</v>
-      </c>
-      <c r="M28" s="23" t="s">
+      <c r="L28" s="22">
+        <v>4</v>
+      </c>
+      <c r="M28" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="N28" s="23" t="s">
+      <c r="N28" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="O28" s="23" t="s">
+      <c r="O28" s="22" t="s">
         <v>72</v>
       </c>
       <c r="P28" s="1" t="s">
@@ -3114,7 +3108,7 @@
       </c>
       <c r="R28" s="1"/>
     </row>
-    <row r="29" spans="1:18" ht="27" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:18" ht="39.9">
       <c r="A29" s="1">
         <v>27</v>
       </c>
@@ -3124,10 +3118,10 @@
       <c r="C29" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D29" s="28" t="s">
+      <c r="D29" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E29" s="23" t="s">
+      <c r="E29" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F29" s="1" t="s">
@@ -3139,25 +3133,25 @@
       <c r="H29" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="I29" s="31" t="s">
+      <c r="I29" s="30" t="s">
         <v>116</v>
       </c>
-      <c r="J29" s="31" t="s">
+      <c r="J29" s="30" t="s">
         <v>223</v>
       </c>
-      <c r="K29" s="23" t="s">
+      <c r="K29" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="L29" s="23">
-        <v>4</v>
-      </c>
-      <c r="M29" s="23" t="s">
+      <c r="L29" s="22">
+        <v>4</v>
+      </c>
+      <c r="M29" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="N29" s="23" t="s">
+      <c r="N29" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="O29" s="23" t="s">
+      <c r="O29" s="22" t="s">
         <v>93</v>
       </c>
       <c r="P29" s="1" t="s">
@@ -3168,7 +3162,7 @@
       </c>
       <c r="R29" s="1"/>
     </row>
-    <row r="30" spans="1:18" ht="27" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:18" ht="39.9">
       <c r="A30" s="1">
         <v>28</v>
       </c>
@@ -3178,10 +3172,10 @@
       <c r="C30" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D30" s="28" t="s">
+      <c r="D30" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E30" s="23" t="s">
+      <c r="E30" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F30" s="1" t="s">
@@ -3193,25 +3187,25 @@
       <c r="H30" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="I30" s="31" t="s">
+      <c r="I30" s="30" t="s">
         <v>116</v>
       </c>
-      <c r="J30" s="31" t="s">
+      <c r="J30" s="30" t="s">
         <v>223</v>
       </c>
-      <c r="K30" s="23" t="s">
+      <c r="K30" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="L30" s="23">
-        <v>4</v>
-      </c>
-      <c r="M30" s="23" t="s">
+      <c r="L30" s="22">
+        <v>4</v>
+      </c>
+      <c r="M30" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="N30" s="23" t="s">
+      <c r="N30" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="O30" s="23" t="s">
+      <c r="O30" s="22" t="s">
         <v>29</v>
       </c>
       <c r="P30" s="1" t="s">
@@ -3222,7 +3216,7 @@
       </c>
       <c r="R30" s="1"/>
     </row>
-    <row r="31" spans="1:18" ht="27" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:18" ht="39.9">
       <c r="A31" s="1">
         <v>29</v>
       </c>
@@ -3232,10 +3226,10 @@
       <c r="C31" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D31" s="28" t="s">
+      <c r="D31" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E31" s="23" t="s">
+      <c r="E31" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F31" s="1" t="s">
@@ -3244,28 +3238,28 @@
       <c r="G31" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="H31" s="21" t="s">
+      <c r="H31" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="I31" s="31" t="s">
+      <c r="I31" s="30" t="s">
         <v>129</v>
       </c>
-      <c r="J31" s="31" t="s">
+      <c r="J31" s="30" t="s">
         <v>223</v>
       </c>
-      <c r="K31" s="23" t="s">
+      <c r="K31" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="L31" s="23">
-        <v>4</v>
-      </c>
-      <c r="M31" s="23" t="s">
+      <c r="L31" s="22">
+        <v>4</v>
+      </c>
+      <c r="M31" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="N31" s="23" t="s">
+      <c r="N31" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="O31" s="23" t="s">
+      <c r="O31" s="22" t="s">
         <v>93</v>
       </c>
       <c r="P31" s="4" t="s">
@@ -3276,7 +3270,7 @@
       </c>
       <c r="R31" s="1"/>
     </row>
-    <row r="32" spans="1:18" ht="27" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:18" ht="39.9">
       <c r="A32" s="1">
         <v>30</v>
       </c>
@@ -3286,10 +3280,10 @@
       <c r="C32" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D32" s="28" t="s">
+      <c r="D32" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E32" s="23" t="s">
+      <c r="E32" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F32" s="1" t="s">
@@ -3301,25 +3295,25 @@
       <c r="H32" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="I32" s="31" t="s">
+      <c r="I32" s="30" t="s">
         <v>116</v>
       </c>
-      <c r="J32" s="31" t="s">
+      <c r="J32" s="30" t="s">
         <v>223</v>
       </c>
-      <c r="K32" s="23" t="s">
+      <c r="K32" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="L32" s="23">
-        <v>4</v>
-      </c>
-      <c r="M32" s="23" t="s">
+      <c r="L32" s="22">
+        <v>4</v>
+      </c>
+      <c r="M32" s="22" t="s">
         <v>147</v>
       </c>
-      <c r="N32" s="23" t="s">
+      <c r="N32" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="O32" s="23" t="s">
+      <c r="O32" s="22" t="s">
         <v>29</v>
       </c>
       <c r="P32" s="4" t="s">
@@ -3330,7 +3324,7 @@
       </c>
       <c r="R32" s="1"/>
     </row>
-    <row r="33" spans="1:18" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:18" ht="39.9">
       <c r="A33" s="1">
         <v>31</v>
       </c>
@@ -3340,10 +3334,10 @@
       <c r="C33" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D33" s="28" t="s">
+      <c r="D33" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E33" s="23" t="s">
+      <c r="E33" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F33" s="1" t="s">
@@ -3355,25 +3349,25 @@
       <c r="H33" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="I33" s="31" t="s">
+      <c r="I33" s="30" t="s">
         <v>116</v>
       </c>
-      <c r="J33" s="31" t="s">
+      <c r="J33" s="30" t="s">
         <v>223</v>
       </c>
-      <c r="K33" s="23" t="s">
+      <c r="K33" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="L33" s="23">
-        <v>4</v>
-      </c>
-      <c r="M33" s="23" t="s">
+      <c r="L33" s="22">
+        <v>4</v>
+      </c>
+      <c r="M33" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="N33" s="23" t="s">
+      <c r="N33" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="O33" s="23" t="s">
+      <c r="O33" s="22" t="s">
         <v>152</v>
       </c>
       <c r="P33" s="4" t="s">
@@ -3384,7 +3378,7 @@
       </c>
       <c r="R33" s="1"/>
     </row>
-    <row r="34" spans="1:18" ht="27" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:18" ht="39.9">
       <c r="A34" s="1">
         <v>32</v>
       </c>
@@ -3394,10 +3388,10 @@
       <c r="C34" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D34" s="28" t="s">
+      <c r="D34" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E34" s="23" t="s">
+      <c r="E34" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F34" s="1" t="s">
@@ -3406,28 +3400,28 @@
       <c r="G34" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="H34" s="21" t="s">
+      <c r="H34" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="I34" s="31" t="s">
+      <c r="I34" s="30" t="s">
         <v>116</v>
       </c>
-      <c r="J34" s="31" t="s">
+      <c r="J34" s="30" t="s">
         <v>223</v>
       </c>
-      <c r="K34" s="23" t="s">
+      <c r="K34" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="L34" s="23">
-        <v>4</v>
-      </c>
-      <c r="M34" s="23" t="s">
+      <c r="L34" s="22">
+        <v>4</v>
+      </c>
+      <c r="M34" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="N34" s="23" t="s">
+      <c r="N34" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="O34" s="23" t="s">
+      <c r="O34" s="22" t="s">
         <v>93</v>
       </c>
       <c r="P34" s="1" t="s">
@@ -3438,7 +3432,7 @@
       </c>
       <c r="R34" s="1"/>
     </row>
-    <row r="35" spans="1:18" ht="27" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:18" ht="39.9">
       <c r="A35" s="1">
         <v>33</v>
       </c>
@@ -3448,10 +3442,10 @@
       <c r="C35" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D35" s="28" t="s">
+      <c r="D35" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E35" s="23" t="s">
+      <c r="E35" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F35" s="1" t="s">
@@ -3463,28 +3457,28 @@
       <c r="H35" s="11" t="s">
         <v>159</v>
       </c>
-      <c r="I35" s="31" t="s">
+      <c r="I35" s="30" t="s">
         <v>129</v>
       </c>
-      <c r="J35" s="31" t="s">
+      <c r="J35" s="30" t="s">
         <v>223</v>
       </c>
-      <c r="K35" s="23" t="s">
+      <c r="K35" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="L35" s="23">
-        <v>4</v>
-      </c>
-      <c r="M35" s="23" t="s">
+      <c r="L35" s="22">
+        <v>4</v>
+      </c>
+      <c r="M35" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="N35" s="23" t="s">
+      <c r="N35" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="O35" s="23" t="s">
+      <c r="O35" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="P35" s="32" t="s">
+      <c r="P35" s="31" t="s">
         <v>160</v>
       </c>
       <c r="Q35" s="15" t="s">
@@ -3492,7 +3486,7 @@
       </c>
       <c r="R35" s="1"/>
     </row>
-    <row r="36" spans="1:18" ht="33" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:18" ht="39.9">
       <c r="A36" s="1">
         <v>34</v>
       </c>
@@ -3502,10 +3496,10 @@
       <c r="C36" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D36" s="28" t="s">
+      <c r="D36" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E36" s="23" t="s">
+      <c r="E36" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F36" s="1" t="s">
@@ -3517,25 +3511,25 @@
       <c r="H36" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="I36" s="31" t="s">
+      <c r="I36" s="30" t="s">
         <v>79</v>
       </c>
-      <c r="J36" s="31" t="s">
+      <c r="J36" s="30" t="s">
         <v>221</v>
       </c>
-      <c r="K36" s="23" t="s">
+      <c r="K36" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="L36" s="23">
-        <v>4</v>
-      </c>
-      <c r="M36" s="23" t="s">
+      <c r="L36" s="22">
+        <v>4</v>
+      </c>
+      <c r="M36" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="N36" s="23" t="s">
+      <c r="N36" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="O36" s="23" t="s">
+      <c r="O36" s="22" t="s">
         <v>29</v>
       </c>
       <c r="P36" s="4" t="s">
@@ -3546,7 +3540,7 @@
       </c>
       <c r="R36" s="1"/>
     </row>
-    <row r="37" spans="1:18" ht="33" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:18" ht="39.9">
       <c r="A37" s="1">
         <v>35</v>
       </c>
@@ -3556,10 +3550,10 @@
       <c r="C37" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D37" s="28" t="s">
+      <c r="D37" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E37" s="23" t="s">
+      <c r="E37" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F37" s="1" t="s">
@@ -3571,25 +3565,25 @@
       <c r="H37" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="I37" s="31" t="s">
+      <c r="I37" s="30" t="s">
         <v>116</v>
       </c>
-      <c r="J37" s="31" t="s">
+      <c r="J37" s="30" t="s">
         <v>223</v>
       </c>
-      <c r="K37" s="23" t="s">
+      <c r="K37" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="L37" s="23">
-        <v>4</v>
-      </c>
-      <c r="M37" s="23" t="s">
+      <c r="L37" s="22">
+        <v>4</v>
+      </c>
+      <c r="M37" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="N37" s="23" t="s">
+      <c r="N37" s="22" t="s">
         <v>167</v>
       </c>
-      <c r="O37" s="23" t="s">
+      <c r="O37" s="22" t="s">
         <v>93</v>
       </c>
       <c r="P37" s="4" t="s">
@@ -3600,7 +3594,7 @@
       </c>
       <c r="R37" s="1"/>
     </row>
-    <row r="38" spans="1:18" ht="27" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:18" ht="39.9">
       <c r="A38" s="1">
         <v>36</v>
       </c>
@@ -3610,10 +3604,10 @@
       <c r="C38" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D38" s="28" t="s">
+      <c r="D38" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E38" s="23" t="s">
+      <c r="E38" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F38" s="1" t="s">
@@ -3625,25 +3619,25 @@
       <c r="H38" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="I38" s="31" t="s">
+      <c r="I38" s="30" t="s">
         <v>116</v>
       </c>
-      <c r="J38" s="31" t="s">
+      <c r="J38" s="30" t="s">
         <v>223</v>
       </c>
-      <c r="K38" s="23" t="s">
+      <c r="K38" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="L38" s="23">
-        <v>4</v>
-      </c>
-      <c r="M38" s="23" t="s">
+      <c r="L38" s="22">
+        <v>4</v>
+      </c>
+      <c r="M38" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="N38" s="23" t="s">
+      <c r="N38" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="O38" s="23" t="s">
+      <c r="O38" s="22" t="s">
         <v>93</v>
       </c>
       <c r="P38" s="4" t="s">
@@ -3654,7 +3648,7 @@
       </c>
       <c r="R38" s="1"/>
     </row>
-    <row r="39" spans="1:18" ht="33" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:18" ht="39.9">
       <c r="A39" s="1">
         <v>37</v>
       </c>
@@ -3664,10 +3658,10 @@
       <c r="C39" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D39" s="28" t="s">
+      <c r="D39" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E39" s="23" t="s">
+      <c r="E39" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F39" s="1" t="s">
@@ -3679,25 +3673,25 @@
       <c r="H39" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="I39" s="31" t="s">
+      <c r="I39" s="30" t="s">
         <v>92</v>
       </c>
-      <c r="J39" s="31" t="s">
+      <c r="J39" s="30" t="s">
         <v>222</v>
       </c>
-      <c r="K39" s="23" t="s">
+      <c r="K39" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="L39" s="23">
-        <v>4</v>
-      </c>
-      <c r="M39" s="23" t="s">
+      <c r="L39" s="22">
+        <v>4</v>
+      </c>
+      <c r="M39" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="N39" s="23" t="s">
+      <c r="N39" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="O39" s="23" t="s">
+      <c r="O39" s="22" t="s">
         <v>93</v>
       </c>
       <c r="P39" s="4" t="s">
@@ -3710,7 +3704,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="40" spans="1:18" ht="27" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:18" ht="39.9">
       <c r="A40" s="1">
         <v>38</v>
       </c>
@@ -3720,10 +3714,10 @@
       <c r="C40" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D40" s="28" t="s">
+      <c r="D40" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E40" s="23" t="s">
+      <c r="E40" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F40" s="1" t="s">
@@ -3735,25 +3729,25 @@
       <c r="H40" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="I40" s="31" t="s">
+      <c r="I40" s="30" t="s">
         <v>92</v>
       </c>
-      <c r="J40" s="31" t="s">
+      <c r="J40" s="30" t="s">
         <v>222</v>
       </c>
-      <c r="K40" s="23" t="s">
+      <c r="K40" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="L40" s="23">
-        <v>4</v>
-      </c>
-      <c r="M40" s="23" t="s">
+      <c r="L40" s="22">
+        <v>4</v>
+      </c>
+      <c r="M40" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="N40" s="23" t="s">
+      <c r="N40" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="O40" s="23" t="s">
+      <c r="O40" s="22" t="s">
         <v>93</v>
       </c>
       <c r="P40" s="4" t="s">
@@ -3764,7 +3758,7 @@
       </c>
       <c r="R40" s="1"/>
     </row>
-    <row r="41" spans="1:18" ht="27" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:18" ht="39.9">
       <c r="A41" s="1">
         <v>39</v>
       </c>
@@ -3774,10 +3768,10 @@
       <c r="C41" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D41" s="28" t="s">
+      <c r="D41" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="E41" s="23" t="s">
+      <c r="E41" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F41" s="1" t="s">
@@ -3789,25 +3783,25 @@
       <c r="H41" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="I41" s="31" t="s">
+      <c r="I41" s="30" t="s">
         <v>103</v>
       </c>
-      <c r="J41" s="31" t="s">
+      <c r="J41" s="30" t="s">
         <v>222</v>
       </c>
-      <c r="K41" s="23" t="s">
+      <c r="K41" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="L41" s="23">
-        <v>4</v>
-      </c>
-      <c r="M41" s="23" t="s">
+      <c r="L41" s="22">
+        <v>4</v>
+      </c>
+      <c r="M41" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="N41" s="23" t="s">
+      <c r="N41" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="O41" s="23" t="s">
+      <c r="O41" s="22" t="s">
         <v>93</v>
       </c>
       <c r="P41" s="4" t="s">
@@ -3876,13 +3870,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66E1BD10-89A3-42E0-BE68-F2421B2B9EE4}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6"/>
   <cols>
-    <col min="1" max="1" width="85.375" customWidth="1"/>
+    <col min="1" max="1" width="85.3828125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="189.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="27" t="s">
+    <row r="1" spans="1:1" ht="189.45">
+      <c r="A1" s="26" t="s">
         <v>217</v>
       </c>
     </row>

</xml_diff>